<commit_message>
Update NBA features + predictions: 2026-10-02 13:52
</commit_message>
<xml_diff>
--- a/nba-backend/data_delivery/nba_feature_workbook_20261002.xlsx
+++ b/nba-backend/data_delivery/nba_feature_workbook_20261002.xlsx
@@ -493,7 +493,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>nba-prod-v2.2-per-side-opp-weighted</t>
+          <t>nba-prod-v2.3-epm</t>
         </is>
       </c>
     </row>
@@ -662,7 +662,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Team features (the trailing-state ladder) and player lines (the position-segmented shrunk TS ratings); assists/rebounds cross-checks against play-by-play.</t>
+          <t>Team features (the trailing-state ladder) and player lines (the position-segmented shrunk EPM ratings); assists/rebounds cross-checks against play-by-play.</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -710,7 +710,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Point-in-time exclusion from the projected lineup pool for the pl_ts_* family (Out/Doubtful/Recovery removed from that game only).</t>
+          <t>Point-in-time exclusion from the projected lineup pool for the pl_epm_* family (Out/Doubtful/Recovery removed from that game only).</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -2018,7 +2018,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Team trailing states and shrunk TS carry the signal; per-player plus-minus is noise-dominated at lineup granularity.</t>
+          <t>Team trailing states and shrunk EPM carry the signal; raw per-player plus-minus is noise-dominated until the EPM family shrinks it per 100 possessions.</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr"/>
@@ -5835,17 +5835,17 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_c_away</t>
+          <t>pl_epm_c_away</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>position-segmented shrunk true-shooting rating of the projected lineup, away side</t>
+          <t>position-segmented shrunk estimated plus-minus of the projected lineup, away side</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk TS -&gt; projected lineup average (official NBA injury report (published designations archive)) (away side)</t>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (away side)</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
@@ -5867,17 +5867,17 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_c_home</t>
+          <t>pl_epm_c_home</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>position-segmented shrunk true-shooting rating of the projected lineup, home side</t>
+          <t>position-segmented shrunk estimated plus-minus of the projected lineup, home side</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk TS -&gt; projected lineup average (official NBA injury report (published designations archive)) (home side)</t>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (home side)</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
@@ -5899,17 +5899,17 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_c_diff</t>
+          <t>pl_epm_c_diff</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>home minus away gap in the position-segmented shrunk true-shooting rating of the projected lineup</t>
+          <t>home minus away gap in the position-segmented shrunk estimated plus-minus of the projected lineup</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk TS -&gt; projected lineup average (official NBA injury report (published designations archive))</t>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive))</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
@@ -5931,17 +5931,17 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_f_away</t>
+          <t>pl_epm_f_away</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>position-segmented shrunk true-shooting rating of the projected lineup, away side</t>
+          <t>position-segmented shrunk estimated plus-minus of the projected lineup, away side</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk TS -&gt; projected lineup average (official NBA injury report (published designations archive)) (away side)</t>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (away side)</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
@@ -5963,17 +5963,17 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_f_home</t>
+          <t>pl_epm_f_home</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>position-segmented shrunk true-shooting rating of the projected lineup, home side</t>
+          <t>position-segmented shrunk estimated plus-minus of the projected lineup, home side</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk TS -&gt; projected lineup average (official NBA injury report (published designations archive)) (home side)</t>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (home side)</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
@@ -5995,17 +5995,17 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_f_diff</t>
+          <t>pl_epm_f_diff</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>home minus away gap in the position-segmented shrunk true-shooting rating of the projected lineup</t>
+          <t>home minus away gap in the position-segmented shrunk estimated plus-minus of the projected lineup</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk TS -&gt; projected lineup average (official NBA injury report (published designations archive))</t>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive))</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
@@ -6027,17 +6027,17 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_g_away</t>
+          <t>pl_epm_g_away</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>position-segmented shrunk true-shooting rating of the projected lineup, away side</t>
+          <t>position-segmented shrunk estimated plus-minus of the projected lineup, away side</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk TS -&gt; projected lineup average (official NBA injury report (published designations archive)) (away side)</t>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (away side)</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
@@ -6059,17 +6059,17 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_g_home</t>
+          <t>pl_epm_g_home</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>position-segmented shrunk true-shooting rating of the projected lineup, home side</t>
+          <t>position-segmented shrunk estimated plus-minus of the projected lineup, home side</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk TS -&gt; projected lineup average (official NBA injury report (published designations archive)) (home side)</t>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (home side)</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
@@ -6091,17 +6091,17 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_g_diff</t>
+          <t>pl_epm_g_diff</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>home minus away gap in the position-segmented shrunk true-shooting rating of the projected lineup</t>
+          <t>home minus away gap in the position-segmented shrunk estimated plus-minus of the projected lineup</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk TS -&gt; projected lineup average (official NBA injury report (published designations archive))</t>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive))</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
@@ -8309,7 +8309,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_c_away</t>
+          <t>pl_epm_c_away</t>
         </is>
       </c>
       <c r="B64" s="2" t="b">
@@ -8322,7 +8322,7 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_c_home</t>
+          <t>pl_epm_c_home</t>
         </is>
       </c>
       <c r="B65" s="2" t="b">
@@ -8335,7 +8335,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_c_diff</t>
+          <t>pl_epm_c_diff</t>
         </is>
       </c>
       <c r="B66" s="2" t="b">
@@ -8348,7 +8348,7 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_f_away</t>
+          <t>pl_epm_f_away</t>
         </is>
       </c>
       <c r="B67" s="2" t="b">
@@ -8361,7 +8361,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_f_home</t>
+          <t>pl_epm_f_home</t>
         </is>
       </c>
       <c r="B68" s="2" t="b">
@@ -8374,7 +8374,7 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_f_diff</t>
+          <t>pl_epm_f_diff</t>
         </is>
       </c>
       <c r="B69" s="2" t="b">
@@ -8387,7 +8387,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_g_away</t>
+          <t>pl_epm_g_away</t>
         </is>
       </c>
       <c r="B70" s="2" t="b">
@@ -8400,7 +8400,7 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_g_home</t>
+          <t>pl_epm_g_home</t>
         </is>
       </c>
       <c r="B71" s="2" t="b">
@@ -8413,7 +8413,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_g_diff</t>
+          <t>pl_epm_g_diff</t>
         </is>
       </c>
       <c r="B72" s="2" t="b">
@@ -9020,7 +9020,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>nba-prod-v2.2-per-side-opp-weighted</t>
+          <t>nba-prod-v2.3-epm</t>
         </is>
       </c>
     </row>
@@ -9356,7 +9356,7 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>78.627</v>
+        <v>67.4284</v>
       </c>
       <c r="C17" s="2" t="n"/>
       <c r="D17" s="2" t="n"/>
@@ -9369,7 +9369,7 @@
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>1.6489</v>
+        <v>1.8333</v>
       </c>
       <c r="C18" s="2" t="n"/>
       <c r="D18" s="2" t="n"/>
@@ -9382,7 +9382,7 @@
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>1.501</v>
+        <v>1.579</v>
       </c>
       <c r="C19" s="2" t="n"/>
       <c r="D19" s="2" t="n"/>
@@ -9395,7 +9395,7 @@
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>1.4148</v>
+        <v>1.4306</v>
       </c>
       <c r="C20" s="2" t="n"/>
       <c r="D20" s="2" t="n"/>
@@ -9408,7 +9408,7 @@
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>0.9686</v>
+        <v>1.1436</v>
       </c>
       <c r="C21" s="2" t="n"/>
       <c r="D21" s="2" t="n"/>
@@ -9421,7 +9421,7 @@
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>0.5421</v>
+        <v>0.9325</v>
       </c>
       <c r="C22" s="2" t="n"/>
       <c r="D22" s="2" t="n"/>
@@ -9430,11 +9430,11 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>ewm_turnover_margin_diff</t>
+          <t>pl_ts_f_diff</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>0.5206</v>
+        <v>0.8923</v>
       </c>
       <c r="C23" s="2" t="n"/>
       <c r="D23" s="2" t="n"/>
@@ -9443,11 +9443,11 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_f_diff</t>
+          <t>elo_home</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>0.52</v>
+        <v>0.8901</v>
       </c>
       <c r="C24" s="2" t="n"/>
       <c r="D24" s="2" t="n"/>
@@ -9456,11 +9456,11 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>elo_home</t>
+          <t>ewm_ast_per_game_diff</t>
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>0.5175</v>
+        <v>0.869</v>
       </c>
       <c r="C25" s="2" t="n"/>
       <c r="D25" s="2" t="n"/>
@@ -9469,11 +9469,11 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>ewm_ast_per_game_diff</t>
+          <t>event_shooting_fouls_away</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>0.5052</v>
+        <v>0.8266</v>
       </c>
       <c r="C26" s="2" t="n"/>
       <c r="D26" s="2" t="n"/>
@@ -9592,7 +9592,7 @@
         <v>100</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>78.627</v>
+        <v>67.4284</v>
       </c>
     </row>
     <row r="3">
@@ -9635,7 +9635,7 @@
         <v>100</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>0.1663</v>
+        <v>0.2861</v>
       </c>
     </row>
     <row r="4">
@@ -9678,7 +9678,7 @@
         <v>100</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>0.4922</v>
+        <v>0.5087</v>
       </c>
     </row>
     <row r="5">
@@ -9721,7 +9721,7 @@
         <v>100</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>0.1272</v>
+        <v>0.167</v>
       </c>
     </row>
     <row r="6">
@@ -9764,7 +9764,7 @@
         <v>100</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>1.6489</v>
+        <v>1.8333</v>
       </c>
     </row>
     <row r="7">
@@ -9807,7 +9807,7 @@
         <v>100</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>1.4148</v>
+        <v>1.4306</v>
       </c>
     </row>
     <row r="8">
@@ -9850,7 +9850,7 @@
         <v>100</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>1.501</v>
+        <v>1.579</v>
       </c>
     </row>
     <row r="9">
@@ -9893,7 +9893,7 @@
         <v>100</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>0.1109</v>
+        <v>0.1907</v>
       </c>
     </row>
     <row r="10">
@@ -9936,7 +9936,7 @@
         <v>100</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>0.2957</v>
+        <v>0.5087</v>
       </c>
     </row>
     <row r="11">
@@ -9979,7 +9979,7 @@
         <v>100</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>0.5206</v>
+        <v>0.7531</v>
       </c>
     </row>
     <row r="12">
@@ -10022,7 +10022,7 @@
         <v>100</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>0.9686</v>
+        <v>1.1436</v>
       </c>
     </row>
     <row r="13">
@@ -10065,7 +10065,7 @@
         <v>100</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>0.5052</v>
+        <v>0.869</v>
       </c>
     </row>
     <row r="14">
@@ -10108,7 +10108,7 @@
         <v>100</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>0.0035</v>
+        <v>0.0029</v>
       </c>
     </row>
     <row r="15">
@@ -10151,7 +10151,7 @@
         <v>100</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>0.5175</v>
+        <v>0.8901</v>
       </c>
     </row>
     <row r="16">
@@ -10194,7 +10194,7 @@
         <v>100</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>0.4312</v>
+        <v>0.7418</v>
       </c>
     </row>
     <row r="17">
@@ -10237,7 +10237,7 @@
         <v>100</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>0.0185</v>
+        <v>0.0318</v>
       </c>
     </row>
     <row r="18">
@@ -10280,7 +10280,7 @@
         <v>100</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>0.0616</v>
+        <v>0.106</v>
       </c>
     </row>
     <row r="19">
@@ -10323,7 +10323,7 @@
         <v>100</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>0.4189</v>
+        <v>0.7206</v>
       </c>
     </row>
     <row r="20">
@@ -10366,7 +10366,7 @@
         <v>100</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>0.3265</v>
+        <v>0.5616</v>
       </c>
     </row>
     <row r="21">
@@ -10409,7 +10409,7 @@
         <v>100</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>0.2526</v>
+        <v>0.4345</v>
       </c>
     </row>
     <row r="22">
@@ -10452,7 +10452,7 @@
         <v>100</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>0.2649</v>
+        <v>0.4557</v>
       </c>
     </row>
     <row r="23">
@@ -10495,7 +10495,7 @@
         <v>100</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>0.1109</v>
+        <v>0.1907</v>
       </c>
     </row>
     <row r="24">
@@ -10581,7 +10581,7 @@
         <v>100</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>0.0554</v>
+        <v>0.0954</v>
       </c>
     </row>
     <row r="26">
@@ -10667,7 +10667,7 @@
         <v>100</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>0.2095</v>
+        <v>0.3603</v>
       </c>
     </row>
     <row r="28">
@@ -10710,7 +10710,7 @@
         <v>100</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>0.0924</v>
+        <v>0.159</v>
       </c>
     </row>
     <row r="29">
@@ -10753,7 +10753,7 @@
         <v>100</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>0.0801</v>
+        <v>0.1378</v>
       </c>
     </row>
     <row r="30">
@@ -10796,7 +10796,7 @@
         <v>100</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>0.117</v>
+        <v>0.2013</v>
       </c>
     </row>
     <row r="31">
@@ -10839,7 +10839,7 @@
         <v>100</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>0.2772</v>
+        <v>0.4769</v>
       </c>
     </row>
     <row r="32">
@@ -10882,7 +10882,7 @@
         <v>100</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>0.4251</v>
+        <v>0.7312</v>
       </c>
     </row>
     <row r="33">
@@ -10925,7 +10925,7 @@
         <v>100</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>0.1417</v>
+        <v>0.2437</v>
       </c>
     </row>
     <row r="34">
@@ -10968,7 +10968,7 @@
         <v>100</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>0.3511</v>
+        <v>0.604</v>
       </c>
     </row>
     <row r="35">
@@ -11011,7 +11011,7 @@
         <v>100</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>0.3142</v>
+        <v>0.5404</v>
       </c>
     </row>
     <row r="36">
@@ -11054,7 +11054,7 @@
         <v>100</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>0.2033</v>
+        <v>0.3497</v>
       </c>
     </row>
     <row r="37">
@@ -11097,7 +11097,7 @@
         <v>100</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>0.1478</v>
+        <v>0.2543</v>
       </c>
     </row>
     <row r="38">
@@ -11140,7 +11140,7 @@
         <v>100</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>0.154</v>
+        <v>0.2649</v>
       </c>
     </row>
     <row r="39">
@@ -11183,7 +11183,7 @@
         <v>100</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>0.0678</v>
+        <v>0.1166</v>
       </c>
     </row>
     <row r="40">
@@ -11226,7 +11226,7 @@
         <v>100</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>0.3327</v>
+        <v>0.5722</v>
       </c>
     </row>
     <row r="41">
@@ -11269,7 +11269,7 @@
         <v>100</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>0.1787</v>
+        <v>0.3073</v>
       </c>
     </row>
     <row r="42">
@@ -11312,7 +11312,7 @@
         <v>100</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>0.1047</v>
+        <v>0.1801</v>
       </c>
     </row>
     <row r="43">
@@ -11355,7 +11355,7 @@
         <v>100</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>0.191</v>
+        <v>0.3285</v>
       </c>
     </row>
     <row r="44">
@@ -11398,7 +11398,7 @@
         <v>100</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>0.4559</v>
+        <v>0.7842</v>
       </c>
     </row>
     <row r="45">
@@ -11441,7 +11441,7 @@
         <v>100</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>0.2464</v>
+        <v>0.4239</v>
       </c>
     </row>
     <row r="46">
@@ -11484,7 +11484,7 @@
         <v>100</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>0.2957</v>
+        <v>0.5087</v>
       </c>
     </row>
     <row r="47">
@@ -11527,7 +11527,7 @@
         <v>100</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>0.117</v>
+        <v>0.2013</v>
       </c>
     </row>
     <row r="48">
@@ -11570,7 +11570,7 @@
         <v>100</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>0.2403</v>
+        <v>0.4133</v>
       </c>
     </row>
     <row r="49">
@@ -11613,7 +11613,7 @@
         <v>100</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>0.1787</v>
+        <v>0.3073</v>
       </c>
     </row>
     <row r="50">
@@ -11656,7 +11656,7 @@
         <v>100</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>0.2279</v>
+        <v>0.3921</v>
       </c>
     </row>
     <row r="51">
@@ -11699,7 +11699,7 @@
         <v>100</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>0.154</v>
+        <v>0.2649</v>
       </c>
     </row>
     <row r="52">
@@ -11742,7 +11742,7 @@
         <v>100</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>0.4805</v>
+        <v>0.8266</v>
       </c>
     </row>
     <row r="53">
@@ -11785,7 +11785,7 @@
         <v>100</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>0.1355</v>
+        <v>0.2331</v>
       </c>
     </row>
     <row r="54">
@@ -11828,7 +11828,7 @@
         <v>100</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>0.1602</v>
+        <v>0.2755</v>
       </c>
     </row>
     <row r="55">
@@ -11914,7 +11914,7 @@
         <v>100</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>0.0493</v>
+        <v>0.0848</v>
       </c>
     </row>
     <row r="57">
@@ -11957,7 +11957,7 @@
         <v>100</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>0.0455</v>
+        <v>0.0762</v>
       </c>
     </row>
     <row r="58">
@@ -12000,7 +12000,7 @@
         <v>100</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>0.3772</v>
+        <v>0.6476</v>
       </c>
     </row>
     <row r="59">
@@ -12043,7 +12043,7 @@
         <v>100</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>0.2095</v>
+        <v>0.3603</v>
       </c>
     </row>
     <row r="60">
@@ -12086,7 +12086,7 @@
         <v>100</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>0.2772</v>
+        <v>0.4769</v>
       </c>
     </row>
     <row r="61">
@@ -12129,7 +12129,7 @@
         <v>100</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>0.2033</v>
+        <v>0.3497</v>
       </c>
     </row>
     <row r="62">
@@ -12172,7 +12172,7 @@
         <v>100</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>0.424</v>
+        <v>0.6228</v>
       </c>
     </row>
     <row r="63">
@@ -12215,13 +12215,13 @@
         <v>100</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>0.1207</v>
+        <v>0.1991</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_c_away</t>
+          <t>pl_epm_c_away</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -12246,25 +12246,29 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>position-segmented shrunk true-shooting rating of the projected lineup, away side</t>
+          <t>position-segmented shrunk estimated plus-minus of the projected lineup, away side</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk TS -&gt; projected lineup average (official NBA injury report (published designations archive)) (away side)</t>
-        </is>
-      </c>
-      <c r="H64" s="2" t="n">
-        <v>90.3</v>
-      </c>
-      <c r="I64" s="2" t="n">
-        <v>0.417</v>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (away side)</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_c_home</t>
+          <t>pl_epm_c_home</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -12289,25 +12293,29 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>position-segmented shrunk true-shooting rating of the projected lineup, home side</t>
+          <t>position-segmented shrunk estimated plus-minus of the projected lineup, home side</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk TS -&gt; projected lineup average (official NBA injury report (published designations archive)) (home side)</t>
-        </is>
-      </c>
-      <c r="H65" s="2" t="n">
-        <v>87.09999999999999</v>
-      </c>
-      <c r="I65" s="2" t="n">
-        <v>0.1787</v>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (home side)</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_c_diff</t>
+          <t>pl_epm_c_diff</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -12332,25 +12340,29 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>home minus away gap in the position-segmented shrunk true-shooting rating of the projected lineup</t>
+          <t>home minus away gap in the position-segmented shrunk estimated plus-minus of the projected lineup</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk TS -&gt; projected lineup average (official NBA injury report (published designations archive))</t>
-        </is>
-      </c>
-      <c r="H66" s="2" t="n">
-        <v>77.40000000000001</v>
-      </c>
-      <c r="I66" s="2" t="n">
-        <v>0.308</v>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive))</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_f_away</t>
+          <t>pl_epm_f_away</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -12375,25 +12387,29 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>position-segmented shrunk true-shooting rating of the projected lineup, away side</t>
+          <t>position-segmented shrunk estimated plus-minus of the projected lineup, away side</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk TS -&gt; projected lineup average (official NBA injury report (published designations archive)) (away side)</t>
-        </is>
-      </c>
-      <c r="H67" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="I67" s="2" t="n">
-        <v>0.5421</v>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (away side)</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_f_home</t>
+          <t>pl_epm_f_home</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -12418,25 +12434,29 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>position-segmented shrunk true-shooting rating of the projected lineup, home side</t>
+          <t>position-segmented shrunk estimated plus-minus of the projected lineup, home side</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk TS -&gt; projected lineup average (official NBA injury report (published designations archive)) (home side)</t>
-        </is>
-      </c>
-      <c r="H68" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="I68" s="2" t="n">
-        <v>0.4506</v>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (home side)</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_f_diff</t>
+          <t>pl_epm_f_diff</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -12461,25 +12481,29 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>home minus away gap in the position-segmented shrunk true-shooting rating of the projected lineup</t>
+          <t>home minus away gap in the position-segmented shrunk estimated plus-minus of the projected lineup</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk TS -&gt; projected lineup average (official NBA injury report (published designations archive))</t>
-        </is>
-      </c>
-      <c r="H69" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="I69" s="2" t="n">
-        <v>0.52</v>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive))</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_g_away</t>
+          <t>pl_epm_g_away</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -12504,25 +12528,29 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>position-segmented shrunk true-shooting rating of the projected lineup, away side</t>
+          <t>position-segmented shrunk estimated plus-minus of the projected lineup, away side</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk TS -&gt; projected lineup average (official NBA injury report (published designations archive)) (away side)</t>
-        </is>
-      </c>
-      <c r="H70" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="I70" s="2" t="n">
-        <v>0.3881</v>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (away side)</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_g_home</t>
+          <t>pl_epm_g_home</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
@@ -12547,25 +12575,29 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>position-segmented shrunk true-shooting rating of the projected lineup, home side</t>
+          <t>position-segmented shrunk estimated plus-minus of the projected lineup, home side</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk TS -&gt; projected lineup average (official NBA injury report (published designations archive)) (home side)</t>
-        </is>
-      </c>
-      <c r="H71" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="I71" s="2" t="n">
-        <v>0.1478</v>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (home side)</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_g_diff</t>
+          <t>pl_epm_g_diff</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -12590,19 +12622,23 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>home minus away gap in the position-segmented shrunk true-shooting rating of the projected lineup</t>
+          <t>home minus away gap in the position-segmented shrunk estimated plus-minus of the projected lineup</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk TS -&gt; projected lineup average (official NBA injury report (published designations archive))</t>
-        </is>
-      </c>
-      <c r="H72" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="I72" s="2" t="n">
-        <v>0.4209</v>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive))</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I72" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="73">
@@ -14692,7 +14728,7 @@
         <v>100</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>78.627</v>
+        <v>67.4284</v>
       </c>
     </row>
     <row r="3">
@@ -14735,7 +14771,7 @@
         <v>100</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>0.1663</v>
+        <v>0.2861</v>
       </c>
     </row>
     <row r="4">
@@ -14778,7 +14814,7 @@
         <v>100</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>0.4922</v>
+        <v>0.5087</v>
       </c>
     </row>
     <row r="5">
@@ -14821,7 +14857,7 @@
         <v>100</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>0.1272</v>
+        <v>0.167</v>
       </c>
     </row>
     <row r="6">
@@ -14864,7 +14900,7 @@
         <v>100</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>1.6489</v>
+        <v>1.8333</v>
       </c>
     </row>
     <row r="7">
@@ -14907,7 +14943,7 @@
         <v>100</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>1.4148</v>
+        <v>1.4306</v>
       </c>
     </row>
     <row r="8">
@@ -14950,7 +14986,7 @@
         <v>100</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>1.501</v>
+        <v>1.579</v>
       </c>
     </row>
     <row r="9">
@@ -14993,7 +15029,7 @@
         <v>100</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>0.1109</v>
+        <v>0.1907</v>
       </c>
     </row>
     <row r="10">
@@ -15036,7 +15072,7 @@
         <v>100</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>0.2957</v>
+        <v>0.5087</v>
       </c>
     </row>
     <row r="11">
@@ -15079,7 +15115,7 @@
         <v>100</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>0.5206</v>
+        <v>0.7531</v>
       </c>
     </row>
     <row r="12">
@@ -15122,7 +15158,7 @@
         <v>100</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>0.9686</v>
+        <v>1.1436</v>
       </c>
     </row>
     <row r="13">
@@ -15165,7 +15201,7 @@
         <v>100</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>0.5052</v>
+        <v>0.869</v>
       </c>
     </row>
     <row r="14">
@@ -15208,7 +15244,7 @@
         <v>100</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>0.0035</v>
+        <v>0.0029</v>
       </c>
     </row>
     <row r="15">
@@ -15251,7 +15287,7 @@
         <v>100</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>0.5175</v>
+        <v>0.8901</v>
       </c>
     </row>
     <row r="16">
@@ -15294,7 +15330,7 @@
         <v>100</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>0.4312</v>
+        <v>0.7418</v>
       </c>
     </row>
     <row r="17">
@@ -15337,7 +15373,7 @@
         <v>100</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>0.0185</v>
+        <v>0.0318</v>
       </c>
     </row>
     <row r="18">
@@ -15380,7 +15416,7 @@
         <v>100</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>0.0616</v>
+        <v>0.106</v>
       </c>
     </row>
     <row r="19">
@@ -15423,7 +15459,7 @@
         <v>100</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>0.4189</v>
+        <v>0.7206</v>
       </c>
     </row>
     <row r="20">
@@ -15466,7 +15502,7 @@
         <v>100</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>0.3265</v>
+        <v>0.5616</v>
       </c>
     </row>
     <row r="21">
@@ -15509,7 +15545,7 @@
         <v>100</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>0.2526</v>
+        <v>0.4345</v>
       </c>
     </row>
     <row r="22">
@@ -15552,7 +15588,7 @@
         <v>100</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>0.2649</v>
+        <v>0.4557</v>
       </c>
     </row>
     <row r="23">
@@ -15595,7 +15631,7 @@
         <v>100</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>0.1109</v>
+        <v>0.1907</v>
       </c>
     </row>
     <row r="24">
@@ -15681,7 +15717,7 @@
         <v>100</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>0.0554</v>
+        <v>0.0954</v>
       </c>
     </row>
     <row r="26">
@@ -15767,7 +15803,7 @@
         <v>100</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>0.2095</v>
+        <v>0.3603</v>
       </c>
     </row>
     <row r="28">
@@ -15810,7 +15846,7 @@
         <v>100</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>0.0924</v>
+        <v>0.159</v>
       </c>
     </row>
     <row r="29">
@@ -15853,7 +15889,7 @@
         <v>100</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>0.0801</v>
+        <v>0.1378</v>
       </c>
     </row>
     <row r="30">
@@ -15896,7 +15932,7 @@
         <v>100</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>0.117</v>
+        <v>0.2013</v>
       </c>
     </row>
     <row r="31">
@@ -15939,7 +15975,7 @@
         <v>100</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>0.2772</v>
+        <v>0.4769</v>
       </c>
     </row>
     <row r="32">
@@ -15982,7 +16018,7 @@
         <v>100</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>0.4251</v>
+        <v>0.7312</v>
       </c>
     </row>
     <row r="33">
@@ -16025,7 +16061,7 @@
         <v>100</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>0.1417</v>
+        <v>0.2437</v>
       </c>
     </row>
     <row r="34">
@@ -16068,7 +16104,7 @@
         <v>100</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>0.3511</v>
+        <v>0.604</v>
       </c>
     </row>
     <row r="35">
@@ -16111,7 +16147,7 @@
         <v>100</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>0.3142</v>
+        <v>0.5404</v>
       </c>
     </row>
     <row r="36">
@@ -16154,7 +16190,7 @@
         <v>100</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>0.2033</v>
+        <v>0.3497</v>
       </c>
     </row>
     <row r="37">
@@ -16197,7 +16233,7 @@
         <v>100</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>0.1478</v>
+        <v>0.2543</v>
       </c>
     </row>
     <row r="38">
@@ -16240,7 +16276,7 @@
         <v>100</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>0.154</v>
+        <v>0.2649</v>
       </c>
     </row>
     <row r="39">
@@ -16283,7 +16319,7 @@
         <v>100</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>0.0678</v>
+        <v>0.1166</v>
       </c>
     </row>
     <row r="40">
@@ -16326,7 +16362,7 @@
         <v>100</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>0.3327</v>
+        <v>0.5722</v>
       </c>
     </row>
     <row r="41">
@@ -16369,7 +16405,7 @@
         <v>100</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>0.1787</v>
+        <v>0.3073</v>
       </c>
     </row>
     <row r="42">
@@ -16412,7 +16448,7 @@
         <v>100</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>0.1047</v>
+        <v>0.1801</v>
       </c>
     </row>
     <row r="43">
@@ -16455,7 +16491,7 @@
         <v>100</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>0.191</v>
+        <v>0.3285</v>
       </c>
     </row>
     <row r="44">
@@ -16498,7 +16534,7 @@
         <v>100</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>0.4559</v>
+        <v>0.7842</v>
       </c>
     </row>
     <row r="45">
@@ -16541,7 +16577,7 @@
         <v>100</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>0.2464</v>
+        <v>0.4239</v>
       </c>
     </row>
     <row r="46">
@@ -16584,7 +16620,7 @@
         <v>100</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>0.2957</v>
+        <v>0.5087</v>
       </c>
     </row>
     <row r="47">
@@ -16627,7 +16663,7 @@
         <v>100</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>0.117</v>
+        <v>0.2013</v>
       </c>
     </row>
     <row r="48">
@@ -16670,7 +16706,7 @@
         <v>100</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>0.2403</v>
+        <v>0.4133</v>
       </c>
     </row>
     <row r="49">
@@ -16713,7 +16749,7 @@
         <v>100</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>0.1787</v>
+        <v>0.3073</v>
       </c>
     </row>
     <row r="50">
@@ -16756,7 +16792,7 @@
         <v>100</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>0.2279</v>
+        <v>0.3921</v>
       </c>
     </row>
     <row r="51">
@@ -16799,7 +16835,7 @@
         <v>100</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>0.154</v>
+        <v>0.2649</v>
       </c>
     </row>
     <row r="52">
@@ -16842,7 +16878,7 @@
         <v>100</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>0.4805</v>
+        <v>0.8266</v>
       </c>
     </row>
     <row r="53">
@@ -16885,7 +16921,7 @@
         <v>100</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>0.1355</v>
+        <v>0.2331</v>
       </c>
     </row>
     <row r="54">
@@ -16928,7 +16964,7 @@
         <v>100</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>0.1602</v>
+        <v>0.2755</v>
       </c>
     </row>
     <row r="55">
@@ -17014,7 +17050,7 @@
         <v>100</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>0.0493</v>
+        <v>0.0848</v>
       </c>
     </row>
     <row r="57">
@@ -17057,7 +17093,7 @@
         <v>100</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>0.0455</v>
+        <v>0.0762</v>
       </c>
     </row>
     <row r="58">
@@ -17100,7 +17136,7 @@
         <v>100</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>0.3772</v>
+        <v>0.6476</v>
       </c>
     </row>
     <row r="59">
@@ -17143,7 +17179,7 @@
         <v>100</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>0.2095</v>
+        <v>0.3603</v>
       </c>
     </row>
     <row r="60">
@@ -17186,7 +17222,7 @@
         <v>100</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>0.2772</v>
+        <v>0.4769</v>
       </c>
     </row>
     <row r="61">
@@ -17229,7 +17265,7 @@
         <v>100</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>0.2033</v>
+        <v>0.3497</v>
       </c>
     </row>
     <row r="62">
@@ -17272,7 +17308,7 @@
         <v>100</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>0.424</v>
+        <v>0.6228</v>
       </c>
     </row>
     <row r="63">
@@ -17315,13 +17351,13 @@
         <v>100</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>0.1207</v>
+        <v>0.1991</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_c_away</t>
+          <t>pl_epm_c_away</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -17346,25 +17382,29 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>position-segmented shrunk true-shooting rating of the projected lineup, away side</t>
+          <t>position-segmented shrunk estimated plus-minus of the projected lineup, away side</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk TS -&gt; projected lineup average (official NBA injury report (published designations archive)) (away side)</t>
-        </is>
-      </c>
-      <c r="H64" s="2" t="n">
-        <v>90.3</v>
-      </c>
-      <c r="I64" s="2" t="n">
-        <v>0.417</v>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (away side)</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_c_home</t>
+          <t>pl_epm_c_home</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -17389,25 +17429,29 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>position-segmented shrunk true-shooting rating of the projected lineup, home side</t>
+          <t>position-segmented shrunk estimated plus-minus of the projected lineup, home side</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk TS -&gt; projected lineup average (official NBA injury report (published designations archive)) (home side)</t>
-        </is>
-      </c>
-      <c r="H65" s="2" t="n">
-        <v>87.09999999999999</v>
-      </c>
-      <c r="I65" s="2" t="n">
-        <v>0.1787</v>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (home side)</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_c_diff</t>
+          <t>pl_epm_c_diff</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -17432,25 +17476,29 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>home minus away gap in the position-segmented shrunk true-shooting rating of the projected lineup</t>
+          <t>home minus away gap in the position-segmented shrunk estimated plus-minus of the projected lineup</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk TS -&gt; projected lineup average (official NBA injury report (published designations archive))</t>
-        </is>
-      </c>
-      <c r="H66" s="2" t="n">
-        <v>77.40000000000001</v>
-      </c>
-      <c r="I66" s="2" t="n">
-        <v>0.308</v>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive))</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_f_away</t>
+          <t>pl_epm_f_away</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -17475,25 +17523,29 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>position-segmented shrunk true-shooting rating of the projected lineup, away side</t>
+          <t>position-segmented shrunk estimated plus-minus of the projected lineup, away side</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk TS -&gt; projected lineup average (official NBA injury report (published designations archive)) (away side)</t>
-        </is>
-      </c>
-      <c r="H67" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="I67" s="2" t="n">
-        <v>0.5421</v>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (away side)</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_f_home</t>
+          <t>pl_epm_f_home</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -17518,25 +17570,29 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>position-segmented shrunk true-shooting rating of the projected lineup, home side</t>
+          <t>position-segmented shrunk estimated plus-minus of the projected lineup, home side</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk TS -&gt; projected lineup average (official NBA injury report (published designations archive)) (home side)</t>
-        </is>
-      </c>
-      <c r="H68" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="I68" s="2" t="n">
-        <v>0.4506</v>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (home side)</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_f_diff</t>
+          <t>pl_epm_f_diff</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -17561,25 +17617,29 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>home minus away gap in the position-segmented shrunk true-shooting rating of the projected lineup</t>
+          <t>home minus away gap in the position-segmented shrunk estimated plus-minus of the projected lineup</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk TS -&gt; projected lineup average (official NBA injury report (published designations archive))</t>
-        </is>
-      </c>
-      <c r="H69" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="I69" s="2" t="n">
-        <v>0.52</v>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive))</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_g_away</t>
+          <t>pl_epm_g_away</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -17604,25 +17664,29 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>position-segmented shrunk true-shooting rating of the projected lineup, away side</t>
+          <t>position-segmented shrunk estimated plus-minus of the projected lineup, away side</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk TS -&gt; projected lineup average (official NBA injury report (published designations archive)) (away side)</t>
-        </is>
-      </c>
-      <c r="H70" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="I70" s="2" t="n">
-        <v>0.3881</v>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (away side)</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_g_home</t>
+          <t>pl_epm_g_home</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
@@ -17647,25 +17711,29 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>position-segmented shrunk true-shooting rating of the projected lineup, home side</t>
+          <t>position-segmented shrunk estimated plus-minus of the projected lineup, home side</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk TS -&gt; projected lineup average (official NBA injury report (published designations archive)) (home side)</t>
-        </is>
-      </c>
-      <c r="H71" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="I71" s="2" t="n">
-        <v>0.1478</v>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (home side)</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_g_diff</t>
+          <t>pl_epm_g_diff</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -17690,19 +17758,23 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>home minus away gap in the position-segmented shrunk true-shooting rating of the projected lineup</t>
+          <t>home minus away gap in the position-segmented shrunk estimated plus-minus of the projected lineup</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk TS -&gt; projected lineup average (official NBA injury report (published designations archive))</t>
-        </is>
-      </c>
-      <c r="H72" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="I72" s="2" t="n">
-        <v>0.4209</v>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive))</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I72" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update NBA features + predictions: 2026-10-02 20:10
</commit_message>
<xml_diff>
--- a/nba-backend/data_delivery/nba_feature_workbook_20261002.xlsx
+++ b/nba-backend/data_delivery/nba_feature_workbook_20261002.xlsx
@@ -493,7 +493,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>nba-prod-v2.3-epm</t>
+          <t>nba-prod-v2.4-epm</t>
         </is>
       </c>
     </row>
@@ -2092,7 +2092,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_c_diff</t>
+          <t>pl_epm_c_diff</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -2116,7 +2116,7 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_c_home</t>
+          <t>pl_epm_c_home</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -2140,7 +2140,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_c_away</t>
+          <t>pl_epm_c_away</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -2188,7 +2188,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_g_away</t>
+          <t>pl_epm_g_away</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -3244,7 +3244,7 @@
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_f_away</t>
+          <t>pl_epm_f_away</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
@@ -3268,7 +3268,7 @@
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_f_home</t>
+          <t>pl_epm_f_home</t>
         </is>
       </c>
       <c r="B113" s="2" t="inlineStr">
@@ -3292,7 +3292,7 @@
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_f_diff</t>
+          <t>pl_epm_f_diff</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
@@ -3340,7 +3340,7 @@
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_g_home</t>
+          <t>pl_epm_g_home</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
@@ -3772,7 +3772,7 @@
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_g_diff</t>
+          <t>pl_epm_g_diff</t>
         </is>
       </c>
       <c r="B134" s="2" t="inlineStr">
@@ -9020,7 +9020,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>nba-prod-v2.3-epm</t>
+          <t>nba-prod-v2.4-epm</t>
         </is>
       </c>
     </row>
@@ -9356,7 +9356,7 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>67.4284</v>
+        <v>75.01819999999999</v>
       </c>
       <c r="C17" s="2" t="n"/>
       <c r="D17" s="2" t="n"/>
@@ -9365,11 +9365,11 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>ewm_net_points_diff</t>
+          <t>pl_epm_f_diff</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>1.8333</v>
+        <v>2.7767</v>
       </c>
       <c r="C18" s="2" t="n"/>
       <c r="D18" s="2" t="n"/>
@@ -9378,11 +9378,11 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>ewm_def_rating_diff</t>
+          <t>pl_epm_g_diff</t>
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>1.579</v>
+        <v>2.5945</v>
       </c>
       <c r="C19" s="2" t="n"/>
       <c r="D19" s="2" t="n"/>
@@ -9391,11 +9391,11 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>ewm_off_rating_diff</t>
+          <t>ewm_net_points_diff</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>1.4306</v>
+        <v>1.595</v>
       </c>
       <c r="C20" s="2" t="n"/>
       <c r="D20" s="2" t="n"/>
@@ -9404,11 +9404,11 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>ewm_rebound_margin_diff</t>
+          <t>ewm_def_rating_diff</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>1.1436</v>
+        <v>1.4804</v>
       </c>
       <c r="C21" s="2" t="n"/>
       <c r="D21" s="2" t="n"/>
@@ -9417,11 +9417,11 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_f_away</t>
+          <t>ewm_off_rating_diff</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>0.9325</v>
+        <v>1.4174</v>
       </c>
       <c r="C22" s="2" t="n"/>
       <c r="D22" s="2" t="n"/>
@@ -9430,11 +9430,11 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_f_diff</t>
+          <t>rest_days_diff</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>0.8923</v>
+        <v>0.7806</v>
       </c>
       <c r="C23" s="2" t="n"/>
       <c r="D23" s="2" t="n"/>
@@ -9443,11 +9443,11 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>elo_home</t>
+          <t>ewm_rebound_margin_diff</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>0.8901</v>
+        <v>0.6405999999999999</v>
       </c>
       <c r="C24" s="2" t="n"/>
       <c r="D24" s="2" t="n"/>
@@ -9456,11 +9456,11 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>ewm_ast_per_game_diff</t>
+          <t>pl_epm_c_home</t>
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>0.869</v>
+        <v>0.5632</v>
       </c>
       <c r="C25" s="2" t="n"/>
       <c r="D25" s="2" t="n"/>
@@ -9469,11 +9469,11 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>event_shooting_fouls_away</t>
+          <t>ewm_ast_per_game_diff</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>0.8266</v>
+        <v>0.5039</v>
       </c>
       <c r="C26" s="2" t="n"/>
       <c r="D26" s="2" t="n"/>
@@ -9592,7 +9592,7 @@
         <v>100</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>67.4284</v>
+        <v>75.01819999999999</v>
       </c>
     </row>
     <row r="3">
@@ -9635,7 +9635,7 @@
         <v>100</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>0.2861</v>
+        <v>0.1603</v>
       </c>
     </row>
     <row r="4">
@@ -9678,7 +9678,7 @@
         <v>100</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>0.5087</v>
+        <v>0.7806</v>
       </c>
     </row>
     <row r="5">
@@ -9721,7 +9721,7 @@
         <v>100</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>0.167</v>
+        <v>0.1838</v>
       </c>
     </row>
     <row r="6">
@@ -9764,7 +9764,7 @@
         <v>100</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>1.8333</v>
+        <v>1.595</v>
       </c>
     </row>
     <row r="7">
@@ -9807,7 +9807,7 @@
         <v>100</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>1.4306</v>
+        <v>1.4174</v>
       </c>
     </row>
     <row r="8">
@@ -9850,7 +9850,7 @@
         <v>100</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>1.579</v>
+        <v>1.4804</v>
       </c>
     </row>
     <row r="9">
@@ -9893,7 +9893,7 @@
         <v>100</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>0.1907</v>
+        <v>0.0573</v>
       </c>
     </row>
     <row r="10">
@@ -9936,7 +9936,7 @@
         <v>100</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>0.5087</v>
+        <v>0.311</v>
       </c>
     </row>
     <row r="11">
@@ -9979,7 +9979,7 @@
         <v>100</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>0.7531</v>
+        <v>0.292</v>
       </c>
     </row>
     <row r="12">
@@ -10022,7 +10022,7 @@
         <v>100</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>1.1436</v>
+        <v>0.6405999999999999</v>
       </c>
     </row>
     <row r="13">
@@ -10065,7 +10065,7 @@
         <v>100</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>0.869</v>
+        <v>0.5039</v>
       </c>
     </row>
     <row r="14">
@@ -10108,7 +10108,7 @@
         <v>100</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>0.0029</v>
+        <v>0.0018</v>
       </c>
     </row>
     <row r="15">
@@ -10151,7 +10151,7 @@
         <v>100</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>0.8901</v>
+        <v>0.3035</v>
       </c>
     </row>
     <row r="16">
@@ -10194,7 +10194,7 @@
         <v>100</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>0.7418</v>
+        <v>0.2748</v>
       </c>
     </row>
     <row r="17">
@@ -10237,7 +10237,7 @@
         <v>100</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>0.0318</v>
+        <v>0.0286</v>
       </c>
     </row>
     <row r="18">
@@ -10280,7 +10280,7 @@
         <v>100</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>0.106</v>
+        <v>0.0687</v>
       </c>
     </row>
     <row r="19">
@@ -10323,7 +10323,7 @@
         <v>100</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>0.7206</v>
+        <v>0.2691</v>
       </c>
     </row>
     <row r="20">
@@ -10366,7 +10366,7 @@
         <v>100</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>0.5616</v>
+        <v>0.1317</v>
       </c>
     </row>
     <row r="21">
@@ -10409,7 +10409,7 @@
         <v>100</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>0.4345</v>
+        <v>0.1947</v>
       </c>
     </row>
     <row r="22">
@@ -10452,7 +10452,7 @@
         <v>100</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>0.4557</v>
+        <v>0.2004</v>
       </c>
     </row>
     <row r="23">
@@ -10495,7 +10495,7 @@
         <v>100</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>0.1907</v>
+        <v>0.1489</v>
       </c>
     </row>
     <row r="24">
@@ -10538,7 +10538,7 @@
         <v>100</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>0</v>
+        <v>0.0057</v>
       </c>
     </row>
     <row r="25">
@@ -10581,7 +10581,7 @@
         <v>100</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>0.0954</v>
+        <v>0.0344</v>
       </c>
     </row>
     <row r="26">
@@ -10667,7 +10667,7 @@
         <v>100</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>0.3603</v>
+        <v>0.1431</v>
       </c>
     </row>
     <row r="28">
@@ -10710,7 +10710,7 @@
         <v>100</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>0.159</v>
+        <v>0.1088</v>
       </c>
     </row>
     <row r="29">
@@ -10753,7 +10753,7 @@
         <v>100</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>0.1378</v>
+        <v>0.0916</v>
       </c>
     </row>
     <row r="30">
@@ -10796,7 +10796,7 @@
         <v>100</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>0.2013</v>
+        <v>0.1661</v>
       </c>
     </row>
     <row r="31">
@@ -10839,7 +10839,7 @@
         <v>100</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>0.4769</v>
+        <v>0.3035</v>
       </c>
     </row>
     <row r="32">
@@ -10882,7 +10882,7 @@
         <v>100</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>0.7312</v>
+        <v>0.3779</v>
       </c>
     </row>
     <row r="33">
@@ -10925,7 +10925,7 @@
         <v>100</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>0.2437</v>
+        <v>0.1775</v>
       </c>
     </row>
     <row r="34">
@@ -10968,7 +10968,7 @@
         <v>100</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>0.604</v>
+        <v>0.2748</v>
       </c>
     </row>
     <row r="35">
@@ -11011,7 +11011,7 @@
         <v>100</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>0.5404</v>
+        <v>0.3207</v>
       </c>
     </row>
     <row r="36">
@@ -11054,7 +11054,7 @@
         <v>100</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>0.3497</v>
+        <v>0.1603</v>
       </c>
     </row>
     <row r="37">
@@ -11097,7 +11097,7 @@
         <v>100</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>0.2543</v>
+        <v>0.1374</v>
       </c>
     </row>
     <row r="38">
@@ -11140,7 +11140,7 @@
         <v>100</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>0.2649</v>
+        <v>0.2176</v>
       </c>
     </row>
     <row r="39">
@@ -11183,7 +11183,7 @@
         <v>100</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>0.1166</v>
+        <v>0.0515</v>
       </c>
     </row>
     <row r="40">
@@ -11226,7 +11226,7 @@
         <v>100</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>0.5722</v>
+        <v>0.2462</v>
       </c>
     </row>
     <row r="41">
@@ -11269,7 +11269,7 @@
         <v>100</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>0.3073</v>
+        <v>0.1775</v>
       </c>
     </row>
     <row r="42">
@@ -11312,7 +11312,7 @@
         <v>100</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>0.1801</v>
+        <v>0.1145</v>
       </c>
     </row>
     <row r="43">
@@ -11355,7 +11355,7 @@
         <v>100</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>0.3285</v>
+        <v>0.2748</v>
       </c>
     </row>
     <row r="44">
@@ -11398,7 +11398,7 @@
         <v>100</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>0.7842</v>
+        <v>0.4352</v>
       </c>
     </row>
     <row r="45">
@@ -11441,7 +11441,7 @@
         <v>100</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>0.4239</v>
+        <v>0.2806</v>
       </c>
     </row>
     <row r="46">
@@ -11484,7 +11484,7 @@
         <v>100</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>0.5087</v>
+        <v>0.3378</v>
       </c>
     </row>
     <row r="47">
@@ -11527,7 +11527,7 @@
         <v>100</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>0.2013</v>
+        <v>0.1374</v>
       </c>
     </row>
     <row r="48">
@@ -11570,7 +11570,7 @@
         <v>100</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>0.4133</v>
+        <v>0.2691</v>
       </c>
     </row>
     <row r="49">
@@ -11613,7 +11613,7 @@
         <v>100</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>0.3073</v>
+        <v>0.1947</v>
       </c>
     </row>
     <row r="50">
@@ -11656,7 +11656,7 @@
         <v>100</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>0.3921</v>
+        <v>0.2806</v>
       </c>
     </row>
     <row r="51">
@@ -11699,7 +11699,7 @@
         <v>100</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>0.2649</v>
+        <v>0.1947</v>
       </c>
     </row>
     <row r="52">
@@ -11742,7 +11742,7 @@
         <v>100</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>0.8266</v>
+        <v>0.4409</v>
       </c>
     </row>
     <row r="53">
@@ -11785,7 +11785,7 @@
         <v>100</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>0.2331</v>
+        <v>0.1202</v>
       </c>
     </row>
     <row r="54">
@@ -11828,7 +11828,7 @@
         <v>100</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>0.2755</v>
+        <v>0.1489</v>
       </c>
     </row>
     <row r="55">
@@ -11914,7 +11914,7 @@
         <v>100</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>0.0848</v>
+        <v>0.07439999999999999</v>
       </c>
     </row>
     <row r="57">
@@ -11957,7 +11957,7 @@
         <v>100</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>0.0762</v>
+        <v>0.0663</v>
       </c>
     </row>
     <row r="58">
@@ -12000,7 +12000,7 @@
         <v>100</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>0.6476</v>
+        <v>0.4142</v>
       </c>
     </row>
     <row r="59">
@@ -12043,7 +12043,7 @@
         <v>100</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>0.3603</v>
+        <v>0.1604</v>
       </c>
     </row>
     <row r="60">
@@ -12086,7 +12086,7 @@
         <v>100</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>0.4769</v>
+        <v>0.229</v>
       </c>
     </row>
     <row r="61">
@@ -12129,7 +12129,7 @@
         <v>100</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>0.3497</v>
+        <v>0.196</v>
       </c>
     </row>
     <row r="62">
@@ -12172,7 +12172,7 @@
         <v>100</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>0.6228</v>
+        <v>0.4215</v>
       </c>
     </row>
     <row r="63">
@@ -12215,7 +12215,7 @@
         <v>100</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>0.1991</v>
+        <v>0.1202</v>
       </c>
     </row>
     <row r="64">
@@ -12254,15 +12254,11 @@
           <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (away side)</t>
         </is>
       </c>
-      <c r="H64" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I64" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="H64" s="2" t="n">
+        <v>90.3</v>
+      </c>
+      <c r="I64" s="2" t="n">
+        <v>0.3254</v>
       </c>
     </row>
     <row r="65">
@@ -12301,15 +12297,11 @@
           <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (home side)</t>
         </is>
       </c>
-      <c r="H65" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I65" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="H65" s="2" t="n">
+        <v>87.09999999999999</v>
+      </c>
+      <c r="I65" s="2" t="n">
+        <v>0.5632</v>
       </c>
     </row>
     <row r="66">
@@ -12348,15 +12340,11 @@
           <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive))</t>
         </is>
       </c>
-      <c r="H66" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I66" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="H66" s="2" t="n">
+        <v>77.40000000000001</v>
+      </c>
+      <c r="I66" s="2" t="n">
+        <v>0.2757</v>
       </c>
     </row>
     <row r="67">
@@ -12395,15 +12383,11 @@
           <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (away side)</t>
         </is>
       </c>
-      <c r="H67" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I67" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="H67" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="I67" s="2" t="n">
+        <v>0.387</v>
       </c>
     </row>
     <row r="68">
@@ -12442,15 +12426,11 @@
           <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (home side)</t>
         </is>
       </c>
-      <c r="H68" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I68" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="H68" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="I68" s="2" t="n">
+        <v>0.4008</v>
       </c>
     </row>
     <row r="69">
@@ -12489,15 +12469,11 @@
           <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive))</t>
         </is>
       </c>
-      <c r="H69" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I69" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="H69" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="I69" s="2" t="n">
+        <v>2.7767</v>
       </c>
     </row>
     <row r="70">
@@ -12536,15 +12512,11 @@
           <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (away side)</t>
         </is>
       </c>
-      <c r="H70" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I70" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="H70" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="I70" s="2" t="n">
+        <v>0.4844</v>
       </c>
     </row>
     <row r="71">
@@ -12583,15 +12555,11 @@
           <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (home side)</t>
         </is>
       </c>
-      <c r="H71" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I71" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="H71" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="I71" s="2" t="n">
+        <v>0.2233</v>
       </c>
     </row>
     <row r="72">
@@ -12630,15 +12598,11 @@
           <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive))</t>
         </is>
       </c>
-      <c r="H72" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I72" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="H72" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="I72" s="2" t="n">
+        <v>2.5945</v>
       </c>
     </row>
     <row r="73">
@@ -14728,7 +14692,7 @@
         <v>100</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>67.4284</v>
+        <v>75.01819999999999</v>
       </c>
     </row>
     <row r="3">
@@ -14771,7 +14735,7 @@
         <v>100</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>0.2861</v>
+        <v>0.1603</v>
       </c>
     </row>
     <row r="4">
@@ -14814,7 +14778,7 @@
         <v>100</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>0.5087</v>
+        <v>0.7806</v>
       </c>
     </row>
     <row r="5">
@@ -14857,7 +14821,7 @@
         <v>100</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>0.167</v>
+        <v>0.1838</v>
       </c>
     </row>
     <row r="6">
@@ -14900,7 +14864,7 @@
         <v>100</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>1.8333</v>
+        <v>1.595</v>
       </c>
     </row>
     <row r="7">
@@ -14943,7 +14907,7 @@
         <v>100</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>1.4306</v>
+        <v>1.4174</v>
       </c>
     </row>
     <row r="8">
@@ -14986,7 +14950,7 @@
         <v>100</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>1.579</v>
+        <v>1.4804</v>
       </c>
     </row>
     <row r="9">
@@ -15029,7 +14993,7 @@
         <v>100</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>0.1907</v>
+        <v>0.0573</v>
       </c>
     </row>
     <row r="10">
@@ -15072,7 +15036,7 @@
         <v>100</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>0.5087</v>
+        <v>0.311</v>
       </c>
     </row>
     <row r="11">
@@ -15115,7 +15079,7 @@
         <v>100</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>0.7531</v>
+        <v>0.292</v>
       </c>
     </row>
     <row r="12">
@@ -15158,7 +15122,7 @@
         <v>100</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>1.1436</v>
+        <v>0.6405999999999999</v>
       </c>
     </row>
     <row r="13">
@@ -15201,7 +15165,7 @@
         <v>100</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>0.869</v>
+        <v>0.5039</v>
       </c>
     </row>
     <row r="14">
@@ -15244,7 +15208,7 @@
         <v>100</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>0.0029</v>
+        <v>0.0018</v>
       </c>
     </row>
     <row r="15">
@@ -15287,7 +15251,7 @@
         <v>100</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>0.8901</v>
+        <v>0.3035</v>
       </c>
     </row>
     <row r="16">
@@ -15330,7 +15294,7 @@
         <v>100</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>0.7418</v>
+        <v>0.2748</v>
       </c>
     </row>
     <row r="17">
@@ -15373,7 +15337,7 @@
         <v>100</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>0.0318</v>
+        <v>0.0286</v>
       </c>
     </row>
     <row r="18">
@@ -15416,7 +15380,7 @@
         <v>100</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>0.106</v>
+        <v>0.0687</v>
       </c>
     </row>
     <row r="19">
@@ -15459,7 +15423,7 @@
         <v>100</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>0.7206</v>
+        <v>0.2691</v>
       </c>
     </row>
     <row r="20">
@@ -15502,7 +15466,7 @@
         <v>100</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>0.5616</v>
+        <v>0.1317</v>
       </c>
     </row>
     <row r="21">
@@ -15545,7 +15509,7 @@
         <v>100</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>0.4345</v>
+        <v>0.1947</v>
       </c>
     </row>
     <row r="22">
@@ -15588,7 +15552,7 @@
         <v>100</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>0.4557</v>
+        <v>0.2004</v>
       </c>
     </row>
     <row r="23">
@@ -15631,7 +15595,7 @@
         <v>100</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>0.1907</v>
+        <v>0.1489</v>
       </c>
     </row>
     <row r="24">
@@ -15674,7 +15638,7 @@
         <v>100</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>0</v>
+        <v>0.0057</v>
       </c>
     </row>
     <row r="25">
@@ -15717,7 +15681,7 @@
         <v>100</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>0.0954</v>
+        <v>0.0344</v>
       </c>
     </row>
     <row r="26">
@@ -15803,7 +15767,7 @@
         <v>100</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>0.3603</v>
+        <v>0.1431</v>
       </c>
     </row>
     <row r="28">
@@ -15846,7 +15810,7 @@
         <v>100</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>0.159</v>
+        <v>0.1088</v>
       </c>
     </row>
     <row r="29">
@@ -15889,7 +15853,7 @@
         <v>100</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>0.1378</v>
+        <v>0.0916</v>
       </c>
     </row>
     <row r="30">
@@ -15932,7 +15896,7 @@
         <v>100</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>0.2013</v>
+        <v>0.1661</v>
       </c>
     </row>
     <row r="31">
@@ -15975,7 +15939,7 @@
         <v>100</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>0.4769</v>
+        <v>0.3035</v>
       </c>
     </row>
     <row r="32">
@@ -16018,7 +15982,7 @@
         <v>100</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>0.7312</v>
+        <v>0.3779</v>
       </c>
     </row>
     <row r="33">
@@ -16061,7 +16025,7 @@
         <v>100</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>0.2437</v>
+        <v>0.1775</v>
       </c>
     </row>
     <row r="34">
@@ -16104,7 +16068,7 @@
         <v>100</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>0.604</v>
+        <v>0.2748</v>
       </c>
     </row>
     <row r="35">
@@ -16147,7 +16111,7 @@
         <v>100</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>0.5404</v>
+        <v>0.3207</v>
       </c>
     </row>
     <row r="36">
@@ -16190,7 +16154,7 @@
         <v>100</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>0.3497</v>
+        <v>0.1603</v>
       </c>
     </row>
     <row r="37">
@@ -16233,7 +16197,7 @@
         <v>100</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>0.2543</v>
+        <v>0.1374</v>
       </c>
     </row>
     <row r="38">
@@ -16276,7 +16240,7 @@
         <v>100</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>0.2649</v>
+        <v>0.2176</v>
       </c>
     </row>
     <row r="39">
@@ -16319,7 +16283,7 @@
         <v>100</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>0.1166</v>
+        <v>0.0515</v>
       </c>
     </row>
     <row r="40">
@@ -16362,7 +16326,7 @@
         <v>100</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>0.5722</v>
+        <v>0.2462</v>
       </c>
     </row>
     <row r="41">
@@ -16405,7 +16369,7 @@
         <v>100</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>0.3073</v>
+        <v>0.1775</v>
       </c>
     </row>
     <row r="42">
@@ -16448,7 +16412,7 @@
         <v>100</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>0.1801</v>
+        <v>0.1145</v>
       </c>
     </row>
     <row r="43">
@@ -16491,7 +16455,7 @@
         <v>100</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>0.3285</v>
+        <v>0.2748</v>
       </c>
     </row>
     <row r="44">
@@ -16534,7 +16498,7 @@
         <v>100</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>0.7842</v>
+        <v>0.4352</v>
       </c>
     </row>
     <row r="45">
@@ -16577,7 +16541,7 @@
         <v>100</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>0.4239</v>
+        <v>0.2806</v>
       </c>
     </row>
     <row r="46">
@@ -16620,7 +16584,7 @@
         <v>100</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>0.5087</v>
+        <v>0.3378</v>
       </c>
     </row>
     <row r="47">
@@ -16663,7 +16627,7 @@
         <v>100</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>0.2013</v>
+        <v>0.1374</v>
       </c>
     </row>
     <row r="48">
@@ -16706,7 +16670,7 @@
         <v>100</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>0.4133</v>
+        <v>0.2691</v>
       </c>
     </row>
     <row r="49">
@@ -16749,7 +16713,7 @@
         <v>100</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>0.3073</v>
+        <v>0.1947</v>
       </c>
     </row>
     <row r="50">
@@ -16792,7 +16756,7 @@
         <v>100</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>0.3921</v>
+        <v>0.2806</v>
       </c>
     </row>
     <row r="51">
@@ -16835,7 +16799,7 @@
         <v>100</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>0.2649</v>
+        <v>0.1947</v>
       </c>
     </row>
     <row r="52">
@@ -16878,7 +16842,7 @@
         <v>100</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>0.8266</v>
+        <v>0.4409</v>
       </c>
     </row>
     <row r="53">
@@ -16921,7 +16885,7 @@
         <v>100</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>0.2331</v>
+        <v>0.1202</v>
       </c>
     </row>
     <row r="54">
@@ -16964,7 +16928,7 @@
         <v>100</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>0.2755</v>
+        <v>0.1489</v>
       </c>
     </row>
     <row r="55">
@@ -17050,7 +17014,7 @@
         <v>100</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>0.0848</v>
+        <v>0.07439999999999999</v>
       </c>
     </row>
     <row r="57">
@@ -17093,7 +17057,7 @@
         <v>100</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>0.0762</v>
+        <v>0.0663</v>
       </c>
     </row>
     <row r="58">
@@ -17136,7 +17100,7 @@
         <v>100</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>0.6476</v>
+        <v>0.4142</v>
       </c>
     </row>
     <row r="59">
@@ -17179,7 +17143,7 @@
         <v>100</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>0.3603</v>
+        <v>0.1604</v>
       </c>
     </row>
     <row r="60">
@@ -17222,7 +17186,7 @@
         <v>100</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>0.4769</v>
+        <v>0.229</v>
       </c>
     </row>
     <row r="61">
@@ -17265,7 +17229,7 @@
         <v>100</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>0.3497</v>
+        <v>0.196</v>
       </c>
     </row>
     <row r="62">
@@ -17308,7 +17272,7 @@
         <v>100</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>0.6228</v>
+        <v>0.4215</v>
       </c>
     </row>
     <row r="63">
@@ -17351,7 +17315,7 @@
         <v>100</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>0.1991</v>
+        <v>0.1202</v>
       </c>
     </row>
     <row r="64">
@@ -17390,15 +17354,11 @@
           <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (away side)</t>
         </is>
       </c>
-      <c r="H64" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I64" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="H64" s="2" t="n">
+        <v>90.3</v>
+      </c>
+      <c r="I64" s="2" t="n">
+        <v>0.3254</v>
       </c>
     </row>
     <row r="65">
@@ -17437,15 +17397,11 @@
           <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (home side)</t>
         </is>
       </c>
-      <c r="H65" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I65" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="H65" s="2" t="n">
+        <v>87.09999999999999</v>
+      </c>
+      <c r="I65" s="2" t="n">
+        <v>0.5632</v>
       </c>
     </row>
     <row r="66">
@@ -17484,15 +17440,11 @@
           <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive))</t>
         </is>
       </c>
-      <c r="H66" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I66" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="H66" s="2" t="n">
+        <v>77.40000000000001</v>
+      </c>
+      <c r="I66" s="2" t="n">
+        <v>0.2757</v>
       </c>
     </row>
     <row r="67">
@@ -17531,15 +17483,11 @@
           <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (away side)</t>
         </is>
       </c>
-      <c r="H67" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I67" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="H67" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="I67" s="2" t="n">
+        <v>0.387</v>
       </c>
     </row>
     <row r="68">
@@ -17578,15 +17526,11 @@
           <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (home side)</t>
         </is>
       </c>
-      <c r="H68" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I68" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="H68" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="I68" s="2" t="n">
+        <v>0.4008</v>
       </c>
     </row>
     <row r="69">
@@ -17625,15 +17569,11 @@
           <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive))</t>
         </is>
       </c>
-      <c r="H69" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I69" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="H69" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="I69" s="2" t="n">
+        <v>2.7767</v>
       </c>
     </row>
     <row r="70">
@@ -17672,15 +17612,11 @@
           <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (away side)</t>
         </is>
       </c>
-      <c r="H70" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I70" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="H70" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="I70" s="2" t="n">
+        <v>0.4844</v>
       </c>
     </row>
     <row r="71">
@@ -17719,15 +17655,11 @@
           <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (home side)</t>
         </is>
       </c>
-      <c r="H71" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I71" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="H71" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="I71" s="2" t="n">
+        <v>0.2233</v>
       </c>
     </row>
     <row r="72">
@@ -17766,15 +17698,11 @@
           <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive))</t>
         </is>
       </c>
-      <c r="H72" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I72" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="H72" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="I72" s="2" t="n">
+        <v>2.5945</v>
       </c>
     </row>
   </sheetData>

</xml_diff>